<commit_message>
Agregado login de seguridad, validacion de fechas y correcion final de la logica de Auto
</commit_message>
<xml_diff>
--- a/concesionaria.xlsx
+++ b/concesionaria.xlsx
@@ -464,17 +464,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mia</t>
+          <t>efef</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>33446453651</t>
+          <t>eef</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>mia@gmail.com</t>
+          <t>efef</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -484,15 +484,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ycs</t>
+          <t>efef</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>570000</v>
+        <v>5545</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Generación de ejecutable .exe, actualización de README y baja lógica en Excel
</commit_message>
<xml_diff>
--- a/concesionaria.xlsx
+++ b/concesionaria.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Ventas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,86 +413,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Teléfono</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Correo</t>
+          <t>Marca</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Marca</t>
+          <t>Modelo</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Modelo</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Precio</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>Fecha</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>efef</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>eef</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>efef</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Ford</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>efef</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>5545</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
         </is>
       </c>
     </row>

</xml_diff>